<commit_message>
data(exemplo): regenera EX-CAMPOBOM-001 com 4pi e caminhos de barra normal
A contraprova de Jacob-Lohman passa de 4,14 (2pi) para 8,29 m3/h, o volume
anual fecha com as linhas em 37.521,84 e os caminhos gravados usam '/', entao o
exemplo abre igual no Linux. As pranchas JPG foram reaproveitadas (--sem-mapas)
para manter a imagem de base da Esri; so o mapa interativo foi redesenhado.
tests/test_exemplo_versionado.py falha se o JSON voltar a ficar para tras.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/processos/EX-CAMPOBOM-001/arquivos/ensaio_bombeamento_PT-01.xlsx
+++ b/data/processos/EX-CAMPOBOM-001/arquivos/ensaio_bombeamento_PT-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Cadastro" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Bombeamento" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Recuperacao" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Orientacoes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="01_Cadastro" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="02_Bombeamento" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="03_Recuperacao" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="04_Orientacoes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>